<commit_message>
menu_auto.py up to date
</commit_message>
<xml_diff>
--- a/menu_sur_6_semaines_RES.xlsx
+++ b/menu_sur_6_semaines_RES.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25601"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE881051-971C-438F-A79D-73A133C90826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1B5B49-0ECE-4871-83B3-DB1CDD704CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="menu_1" sheetId="7" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="344">
   <si>
     <t>semaine</t>
   </si>
@@ -1053,13 +1053,16 @@
     <t xml:space="preserve">soupe aux lentilles et au curry </t>
   </si>
   <si>
-    <t>m/j/aaaa</t>
-  </si>
-  <si>
-    <t>9/5/2022</t>
-  </si>
-  <si>
-    <t>9/12/2022</t>
+    <t>9-19-2022</t>
+  </si>
+  <si>
+    <t>9-12-2022</t>
+  </si>
+  <si>
+    <t>9-5-2022</t>
+  </si>
+  <si>
+    <t>m-j-aaaa</t>
   </si>
 </sst>
 </file>
@@ -1725,7 +1728,7 @@
     </row>
     <row r="2" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" s="32" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B2" s="17">
         <v>22</v>
@@ -1751,7 +1754,7 @@
     </row>
     <row r="3" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>
@@ -2543,7 +2546,7 @@
     </row>
     <row r="3" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>
@@ -3335,7 +3338,7 @@
     </row>
     <row r="3" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>
@@ -4101,7 +4104,7 @@
     </row>
     <row r="2" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" s="32" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B2" s="17">
         <v>22</v>
@@ -4127,7 +4130,7 @@
     </row>
     <row r="3" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>
@@ -4893,7 +4896,7 @@
     </row>
     <row r="2" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" s="32" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B2" s="17">
         <v>22</v>
@@ -4919,7 +4922,7 @@
     </row>
     <row r="3" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>
@@ -5688,7 +5691,7 @@
     </row>
     <row r="2" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" s="32" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B2" s="17">
         <v>22</v>
@@ -5714,7 +5717,7 @@
     </row>
     <row r="3" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>

</xml_diff>